<commit_message>
ptj-internal-estimate: formula model + 現地SV費 auto SV-MD + compact template
- §3 now formula-driven: K26=EBIT input, L26==J26/(1-K26), N26=Offer price input
- total start clears C~I (pre-총원가 columns)
- §4 SV-MD auto-read from 現地SV費 (実働=契約MD, 移動=見積MD−契約MD, SV A–F),
  total C-MD → D7=G37 → L24=220×days
- new --offer flag; compact layout (removed empty-row gap)
- template rebuilt from user's hand-tuned sheet; old kept locally as *.OLD.xlsx

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ptj-internal-estimate/assets/nemae_template.xlsx
+++ b/ptj-internal-estimate/assets/nemae_template.xlsx
@@ -22,7 +22,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="#,##0_ "/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,8 +130,14 @@
       <color rgb="FF0070C0"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Malgun Gothic"/>
+      <charset val="129"/>
+      <family val="3"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -162,14 +168,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="17">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -374,12 +374,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -682,18 +681,12 @@
     <xf numFmtId="167" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="38" fontId="2" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="40" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="40" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="38" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="38" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -712,39 +705,15 @@
     <xf numFmtId="38" fontId="3" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="16" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="16" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="16" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="40" fontId="2" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="38" fontId="3" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="38" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -752,21 +721,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="40" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="3" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
@@ -1150,8 +1112,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AC55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="12.75"/>
+  <dimension ref="A1:AC46"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="13.5"/>
   <cols>
     <col width="3.625" customWidth="1" min="1" max="1"/>
     <col width="18.625" customWidth="1" min="2" max="2"/>
@@ -1159,10 +1121,10 @@
     <col width="10.125" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="11.125" customWidth="1" min="6" max="6"/>
-    <col width="11.125" customWidth="1" min="7" max="7"/>
-    <col width="11.125" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
     <col width="12.5" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="9.25" customWidth="1" min="13" max="13"/>
     <col width="13.625" customWidth="1" min="14" max="14"/>
     <col width="15.25" customWidth="1" min="16" max="16"/>
     <col width="14" customWidth="1" min="17" max="17"/>
@@ -1312,7 +1274,7 @@
         </is>
       </c>
       <c r="J5" s="31" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="K5" s="30" t="inlineStr">
         <is>
@@ -1355,7 +1317,7 @@
         </is>
       </c>
       <c r="J6" s="31" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="K6" s="30" t="n"/>
       <c r="L6" s="30" t="n"/>
@@ -1381,14 +1343,17 @@
     <row r="7" ht="12" customHeight="1">
       <c r="B7" s="37" t="inlineStr">
         <is>
-          <t>Mech</t>
+          <t>SV</t>
         </is>
       </c>
       <c r="C7" s="38">
         <f>D7/D5</f>
         <v/>
       </c>
-      <c r="D7" s="39" t="n"/>
+      <c r="D7" s="39">
+        <f>G37</f>
+        <v/>
+      </c>
       <c r="E7" s="40" t="n"/>
       <c r="F7" s="40" t="n"/>
       <c r="G7" s="41" t="n"/>
@@ -1398,7 +1363,7 @@
         </is>
       </c>
       <c r="J7" s="31" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="K7" s="30" t="n"/>
       <c r="L7" s="30" t="n"/>
@@ -1422,15 +1387,8 @@
       <c r="AC7" s="18" t="n"/>
     </row>
     <row r="8" ht="12" customHeight="1">
-      <c r="B8" s="43" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="C8" s="44">
-        <f>D8/30.5</f>
-        <v/>
-      </c>
+      <c r="B8" s="43" t="n"/>
+      <c r="C8" s="44" t="n"/>
       <c r="D8" s="45" t="n"/>
       <c r="E8" s="46" t="n"/>
       <c r="F8" s="46" t="n"/>
@@ -1568,13 +1526,9 @@
         </is>
       </c>
       <c r="J12" s="62" t="n">
-        <v>120</v>
-      </c>
-      <c r="K12" s="56" t="inlineStr">
-        <is>
-          <t>2023,2024 Korea average</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K12" s="56" t="n"/>
       <c r="L12" s="56" t="n"/>
       <c r="M12" s="56" t="n"/>
       <c r="R12" s="8" t="n"/>
@@ -1602,13 +1556,9 @@
         </is>
       </c>
       <c r="J13" s="66" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="K13" s="56" t="inlineStr">
-        <is>
-          <t>2023,2024 Korea average</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K13" s="56" t="n"/>
       <c r="L13" s="65" t="n"/>
       <c r="M13" s="48" t="n"/>
       <c r="R13" s="8" t="n"/>
@@ -1636,7 +1586,7 @@
         </is>
       </c>
       <c r="J14" s="69" t="n">
-        <v>0.12</v>
+        <v>0</v>
       </c>
       <c r="K14" s="70" t="n"/>
       <c r="L14" s="49" t="n"/>
@@ -1912,19 +1862,10 @@
       <c r="C22" s="99" t="n"/>
       <c r="D22" s="99" t="n"/>
       <c r="E22" s="100" t="n"/>
-      <c r="F22" s="100">
-        <f>$J$8</f>
-        <v/>
-      </c>
-      <c r="G22" s="100">
-        <f>$J$18</f>
-        <v/>
-      </c>
+      <c r="F22" s="100" t="n"/>
+      <c r="G22" s="100" t="n"/>
       <c r="H22" s="99" t="n"/>
-      <c r="I22" s="100">
-        <f>$J$14</f>
-        <v/>
-      </c>
+      <c r="I22" s="100" t="n"/>
       <c r="J22" s="99" t="n"/>
       <c r="K22" s="100">
         <f>K26</f>
@@ -1945,33 +1886,18 @@
       <c r="A23" s="15" t="n"/>
       <c r="B23" s="92" t="inlineStr">
         <is>
-          <t>HWあり</t>
-        </is>
-      </c>
-      <c r="C23" s="102" t="n"/>
+          <t>機械</t>
+        </is>
+      </c>
+      <c r="C23" s="46" t="n"/>
       <c r="D23" s="46" t="n"/>
       <c r="E23" s="46" t="n"/>
-      <c r="F23" s="46">
-        <f>L23*$J$8</f>
-        <v/>
-      </c>
-      <c r="G23" s="46">
-        <f>N23*$G$22</f>
-        <v/>
-      </c>
-      <c r="H23" s="46">
-        <f>SUM(C23:G23)</f>
-        <v/>
-      </c>
-      <c r="I23" s="46">
-        <f>L23*$I$22</f>
-        <v/>
-      </c>
-      <c r="J23" s="46">
-        <f>H23+I23</f>
-        <v/>
-      </c>
-      <c r="K23" s="103">
+      <c r="F23" s="46" t="n"/>
+      <c r="G23" s="46" t="n"/>
+      <c r="H23" s="46" t="n"/>
+      <c r="I23" s="46" t="n"/>
+      <c r="J23" s="46" t="n"/>
+      <c r="K23" s="102">
         <f>(L23-J23)/L23%</f>
         <v/>
       </c>
@@ -1987,7 +1913,7 @@
         <f>N26-N24-N25</f>
         <v/>
       </c>
-      <c r="O23" s="104" t="n"/>
+      <c r="O23" s="103" t="n"/>
       <c r="T23" s="8" t="n"/>
       <c r="AB23" s="8" t="n"/>
       <c r="AC23" s="8" t="n"/>
@@ -1999,40 +1925,19 @@
           <t>SV</t>
         </is>
       </c>
-      <c r="C24" s="102" t="n"/>
-      <c r="D24" s="46">
-        <f>J12*C11</f>
-        <v/>
-      </c>
-      <c r="E24" s="46">
-        <f>L24*J13</f>
-        <v/>
-      </c>
-      <c r="F24" s="46">
-        <f>L24*$J$5</f>
-        <v/>
-      </c>
-      <c r="G24" s="46">
-        <f>N24*$G$22</f>
-        <v/>
-      </c>
-      <c r="H24" s="46">
-        <f>SUM(C24:G24)</f>
-        <v/>
-      </c>
-      <c r="I24" s="46">
-        <f>L24*$I$22</f>
-        <v/>
-      </c>
-      <c r="J24" s="46">
-        <f>H24+I24</f>
-        <v/>
-      </c>
-      <c r="K24" s="103">
+      <c r="C24" s="46" t="n"/>
+      <c r="D24" s="46" t="n"/>
+      <c r="E24" s="46" t="n"/>
+      <c r="F24" s="46" t="n"/>
+      <c r="G24" s="46" t="n"/>
+      <c r="H24" s="46" t="n"/>
+      <c r="I24" s="46" t="n"/>
+      <c r="J24" s="46" t="n"/>
+      <c r="K24" s="102">
         <f>(L24-J24)/L24%</f>
         <v/>
       </c>
-      <c r="L24" s="105">
+      <c r="L24" s="46">
         <f>D16*D11</f>
         <v/>
       </c>
@@ -2040,7 +1945,7 @@
         <f>(N24-L24)/N24</f>
         <v/>
       </c>
-      <c r="N24" s="106">
+      <c r="N24" s="104">
         <f>L24</f>
         <v/>
       </c>
@@ -2056,21 +1961,18 @@
           <t>推奨予備品</t>
         </is>
       </c>
-      <c r="C25" s="106" t="n"/>
-      <c r="D25" s="106" t="n"/>
-      <c r="E25" s="106" t="n"/>
+      <c r="C25" s="104" t="n"/>
+      <c r="D25" s="104" t="n"/>
+      <c r="E25" s="104" t="n"/>
       <c r="F25" s="46" t="n"/>
-      <c r="G25" s="46">
-        <f>N25*$G$22</f>
-        <v/>
-      </c>
+      <c r="G25" s="46" t="n"/>
       <c r="H25" s="46" t="n"/>
       <c r="I25" s="46" t="n"/>
       <c r="J25" s="46" t="n"/>
-      <c r="K25" s="103" t="n"/>
-      <c r="L25" s="105" t="n"/>
+      <c r="K25" s="102" t="n"/>
+      <c r="L25" s="46" t="n"/>
       <c r="M25" s="100" t="n"/>
-      <c r="N25" s="107" t="n"/>
+      <c r="N25" s="105" t="n"/>
       <c r="O25" s="17" t="n"/>
       <c r="T25" s="8" t="n"/>
       <c r="AB25" s="8" t="n"/>
@@ -2083,48 +1985,29 @@
           <t xml:space="preserve">  Total</t>
         </is>
       </c>
-      <c r="C26" s="108">
-        <f>SUM(C23:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="108">
-        <f>SUM(D23:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="108">
-        <f>SUM(E23:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="108">
-        <f>SUM(F23:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="108">
-        <f>SUM(G23:G24)</f>
-        <v/>
-      </c>
-      <c r="H26" s="108">
-        <f>SUM(H23:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="108">
-        <f>SUM(I23:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="108">
+      <c r="C26" s="106" t="n"/>
+      <c r="D26" s="106" t="n"/>
+      <c r="E26" s="106" t="n"/>
+      <c r="F26" s="106" t="n"/>
+      <c r="G26" s="106" t="n"/>
+      <c r="H26" s="106" t="n"/>
+      <c r="I26" s="106" t="n"/>
+      <c r="J26" s="106">
         <f>SUM(J23:J25)</f>
         <v/>
       </c>
-      <c r="K26" s="103">
-        <f>(L26-J26)/L26</f>
-        <v/>
-      </c>
-      <c r="L26" s="109" t="n"/>
-      <c r="M26" s="108">
+      <c r="K26" s="102" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="L26" s="106">
+        <f>J26/(1-K26)</f>
+        <v/>
+      </c>
+      <c r="M26" s="106">
         <f>N26-L26</f>
         <v/>
       </c>
-      <c r="N26" s="109" t="n"/>
+      <c r="N26" s="107" t="n"/>
       <c r="O26" s="17" t="n"/>
       <c r="T26" s="8" t="n"/>
       <c r="AB26" s="8" t="n"/>
@@ -2132,657 +2015,427 @@
     </row>
     <row r="27" ht="12" customHeight="1">
       <c r="A27" s="15" t="n"/>
-      <c r="B27" s="110" t="n"/>
-      <c r="C27" s="111" t="n"/>
-      <c r="D27" s="111" t="n"/>
-      <c r="E27" s="111" t="n"/>
-      <c r="F27" s="111" t="n"/>
-      <c r="G27" s="111" t="n"/>
-      <c r="H27" s="111" t="n"/>
-      <c r="I27" s="111" t="n"/>
-      <c r="J27" s="111" t="n"/>
-      <c r="K27" s="111" t="n"/>
-      <c r="L27" s="111" t="n"/>
-      <c r="M27" s="111" t="n"/>
-      <c r="N27" s="111" t="n"/>
+      <c r="B27" s="108" t="n"/>
+      <c r="C27" s="109" t="n"/>
+      <c r="D27" s="109" t="n"/>
+      <c r="E27" s="109" t="n"/>
+      <c r="F27" s="109" t="n"/>
+      <c r="G27" s="109" t="n"/>
+      <c r="H27" s="109" t="n"/>
+      <c r="I27" s="109" t="n"/>
+      <c r="J27" s="109" t="n"/>
+      <c r="K27" s="109" t="n"/>
+      <c r="L27" s="109" t="n"/>
+      <c r="M27" s="109" t="n"/>
+      <c r="N27" s="109" t="n"/>
       <c r="O27" s="17" t="n"/>
       <c r="T27" s="8" t="n"/>
       <c r="AB27" s="8" t="n"/>
       <c r="AC27" s="8" t="n"/>
     </row>
-    <row r="28" ht="12" customHeight="1">
-      <c r="A28" s="112" t="n"/>
-      <c r="B28" s="112" t="n"/>
-      <c r="C28" s="113" t="n"/>
-      <c r="D28" s="113" t="n"/>
-      <c r="E28" s="114" t="n"/>
-      <c r="F28" s="114" t="n"/>
-      <c r="G28" s="114" t="n"/>
-      <c r="H28" s="113" t="n"/>
-      <c r="I28" s="114" t="n"/>
-      <c r="J28" s="113" t="n"/>
-      <c r="K28" s="114" t="n"/>
-      <c r="L28" s="115" t="n"/>
-      <c r="M28" s="114" t="n"/>
-      <c r="N28" s="116" t="n"/>
-      <c r="O28" s="117" t="n"/>
-      <c r="P28" s="117" t="n"/>
-      <c r="Q28" s="117" t="n"/>
-      <c r="R28" s="117" t="n"/>
-      <c r="S28" s="117" t="n"/>
-      <c r="T28" s="117" t="n"/>
-      <c r="U28" s="117" t="n"/>
-      <c r="V28" s="117" t="n"/>
-      <c r="W28" s="117" t="n"/>
-      <c r="X28" s="117" t="n"/>
-      <c r="Y28" s="117" t="n"/>
-      <c r="Z28" s="117" t="n"/>
-      <c r="AA28" s="117" t="n"/>
-      <c r="AB28" s="117" t="n"/>
-      <c r="AC28" s="117" t="n"/>
-    </row>
-    <row r="29" ht="12" customHeight="1">
-      <c r="A29" s="112" t="n"/>
-      <c r="B29" s="118" t="n"/>
-      <c r="C29" s="119" t="n"/>
-      <c r="D29" s="119" t="n"/>
-      <c r="E29" s="119" t="n"/>
-      <c r="F29" s="119" t="n"/>
-      <c r="G29" s="119" t="n"/>
-      <c r="H29" s="119" t="n"/>
-      <c r="I29" s="119" t="n"/>
-      <c r="J29" s="119" t="n"/>
-      <c r="K29" s="119" t="n"/>
-      <c r="L29" s="119" t="n"/>
-      <c r="M29" s="119" t="n"/>
-      <c r="N29" s="119" t="n"/>
-      <c r="O29" s="120" t="n"/>
-      <c r="P29" s="117" t="n"/>
-      <c r="Q29" s="117" t="n"/>
-      <c r="R29" s="117" t="n"/>
-      <c r="S29" s="117" t="n"/>
-      <c r="T29" s="117" t="n"/>
-      <c r="U29" s="117" t="n"/>
-      <c r="V29" s="117" t="n"/>
-      <c r="W29" s="117" t="n"/>
-      <c r="X29" s="117" t="n"/>
-      <c r="Y29" s="117" t="n"/>
-      <c r="Z29" s="117" t="n"/>
-      <c r="AA29" s="117" t="n"/>
-      <c r="AB29" s="117" t="n"/>
-      <c r="AC29" s="117" t="n"/>
-    </row>
-    <row r="30" ht="12" customHeight="1">
-      <c r="A30" s="112" t="n"/>
-      <c r="B30" s="118" t="n"/>
-      <c r="C30" s="119" t="n"/>
-      <c r="D30" s="119" t="n"/>
-      <c r="E30" s="119" t="n"/>
-      <c r="F30" s="119" t="n"/>
-      <c r="G30" s="119" t="n"/>
-      <c r="H30" s="119" t="n"/>
-      <c r="I30" s="119" t="n"/>
-      <c r="J30" s="119" t="n"/>
-      <c r="K30" s="119" t="n"/>
-      <c r="L30" s="119" t="n"/>
-      <c r="M30" s="119" t="n"/>
-      <c r="N30" s="119" t="n"/>
-      <c r="O30" s="119" t="n"/>
-      <c r="P30" s="117" t="n"/>
-      <c r="Q30" s="117" t="n"/>
-      <c r="R30" s="117" t="n"/>
-      <c r="S30" s="117" t="n"/>
-      <c r="T30" s="117" t="n"/>
-      <c r="U30" s="117" t="n"/>
-      <c r="V30" s="117" t="n"/>
-      <c r="W30" s="117" t="n"/>
-      <c r="X30" s="117" t="n"/>
-      <c r="Y30" s="117" t="n"/>
-      <c r="Z30" s="117" t="n"/>
-      <c r="AA30" s="117" t="n"/>
-      <c r="AB30" s="117" t="n"/>
-      <c r="AC30" s="117" t="n"/>
-    </row>
-    <row r="31" ht="12" customHeight="1">
-      <c r="A31" s="112" t="n"/>
-      <c r="B31" s="112" t="n"/>
-      <c r="C31" s="121" t="n"/>
-      <c r="D31" s="121" t="n"/>
-      <c r="E31" s="121" t="n"/>
-      <c r="F31" s="121" t="n"/>
-      <c r="G31" s="121" t="n"/>
-      <c r="H31" s="121" t="n"/>
-      <c r="I31" s="121" t="n"/>
-      <c r="J31" s="121" t="n"/>
-      <c r="K31" s="121" t="n"/>
-      <c r="L31" s="121" t="n"/>
-      <c r="M31" s="121" t="n"/>
-      <c r="N31" s="121" t="n"/>
-      <c r="O31" s="119" t="n"/>
-      <c r="P31" s="117" t="n"/>
-      <c r="Q31" s="117" t="n"/>
-      <c r="R31" s="117" t="n"/>
-      <c r="S31" s="117" t="n"/>
-      <c r="T31" s="117" t="n"/>
-      <c r="U31" s="117" t="n"/>
-      <c r="V31" s="117" t="n"/>
-      <c r="W31" s="117" t="n"/>
-      <c r="X31" s="117" t="n"/>
-      <c r="Y31" s="117" t="n"/>
-      <c r="Z31" s="117" t="n"/>
-      <c r="AA31" s="117" t="n"/>
-      <c r="AB31" s="117" t="n"/>
-      <c r="AC31" s="117" t="n"/>
-    </row>
-    <row r="32" ht="12" customHeight="1">
-      <c r="A32" s="112" t="n"/>
-      <c r="B32" s="117" t="n"/>
-      <c r="C32" s="121" t="n"/>
-      <c r="D32" s="121" t="n"/>
-      <c r="E32" s="121" t="n"/>
-      <c r="F32" s="121" t="n"/>
-      <c r="G32" s="121" t="n"/>
-      <c r="H32" s="121" t="n"/>
-      <c r="I32" s="121" t="n"/>
-      <c r="J32" s="121" t="n"/>
-      <c r="K32" s="121" t="n"/>
-      <c r="L32" s="121" t="n"/>
-      <c r="M32" s="121" t="n"/>
-      <c r="N32" s="121" t="n"/>
-      <c r="O32" s="119" t="n"/>
-      <c r="P32" s="117" t="n"/>
-      <c r="Q32" s="117" t="n"/>
-      <c r="R32" s="117" t="n"/>
-      <c r="S32" s="117" t="n"/>
-      <c r="T32" s="117" t="n"/>
-      <c r="U32" s="117" t="n"/>
-      <c r="V32" s="117" t="n"/>
-      <c r="W32" s="117" t="n"/>
-      <c r="X32" s="117" t="n"/>
-      <c r="Y32" s="117" t="n"/>
-      <c r="Z32" s="117" t="n"/>
-      <c r="AA32" s="117" t="n"/>
-      <c r="AB32" s="117" t="n"/>
-      <c r="AC32" s="117" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="117" t="n"/>
-      <c r="B33" s="112" t="n"/>
-      <c r="C33" s="113" t="n"/>
-      <c r="D33" s="113" t="n"/>
-      <c r="E33" s="114" t="n"/>
-      <c r="F33" s="114" t="n"/>
-      <c r="G33" s="114" t="n"/>
-      <c r="H33" s="113" t="n"/>
-      <c r="I33" s="114" t="n"/>
-      <c r="J33" s="113" t="n"/>
-      <c r="K33" s="114" t="n"/>
-      <c r="L33" s="115" t="n"/>
-      <c r="M33" s="114" t="n"/>
-      <c r="N33" s="116" t="n"/>
-      <c r="O33" s="119" t="n"/>
-      <c r="P33" s="117" t="n"/>
-      <c r="Q33" s="117" t="n"/>
-      <c r="R33" s="117" t="n"/>
-      <c r="S33" s="119" t="n"/>
-      <c r="T33" s="117" t="n"/>
-      <c r="U33" s="117" t="n"/>
-      <c r="V33" s="117" t="n"/>
-      <c r="W33" s="117" t="n"/>
-      <c r="X33" s="117" t="n"/>
-      <c r="Y33" s="117" t="n"/>
-      <c r="Z33" s="117" t="n"/>
-      <c r="AA33" s="119" t="n"/>
-      <c r="AB33" s="119" t="n"/>
-      <c r="AC33" s="117" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="117" t="n"/>
-      <c r="B34" s="118" t="n"/>
-      <c r="C34" s="119" t="n"/>
-      <c r="D34" s="119" t="n"/>
-      <c r="E34" s="119" t="n"/>
-      <c r="F34" s="119" t="n"/>
-      <c r="G34" s="119" t="n"/>
-      <c r="H34" s="119" t="n"/>
-      <c r="I34" s="119" t="n"/>
-      <c r="J34" s="119" t="n"/>
-      <c r="K34" s="119" t="n"/>
-      <c r="L34" s="119" t="n"/>
-      <c r="M34" s="119" t="n"/>
-      <c r="N34" s="119" t="n"/>
-      <c r="O34" s="119" t="n"/>
-      <c r="P34" s="117" t="n"/>
-      <c r="Q34" s="117" t="n"/>
-      <c r="R34" s="117" t="n"/>
-      <c r="S34" s="119" t="n"/>
-      <c r="T34" s="117" t="n"/>
-      <c r="U34" s="117" t="n"/>
-      <c r="V34" s="117" t="n"/>
-      <c r="W34" s="117" t="n"/>
-      <c r="X34" s="117" t="n"/>
-      <c r="Y34" s="117" t="n"/>
-      <c r="Z34" s="117" t="n"/>
-      <c r="AA34" s="119" t="n"/>
-      <c r="AB34" s="119" t="n"/>
-      <c r="AC34" s="117" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="117" t="n"/>
-      <c r="B35" s="118" t="n"/>
-      <c r="C35" s="119" t="n"/>
-      <c r="D35" s="119" t="n"/>
-      <c r="E35" s="119" t="n"/>
-      <c r="F35" s="119" t="n"/>
-      <c r="G35" s="119" t="n"/>
-      <c r="H35" s="119" t="n"/>
-      <c r="I35" s="119" t="n"/>
-      <c r="J35" s="119" t="n"/>
-      <c r="K35" s="119" t="n"/>
-      <c r="L35" s="119" t="n"/>
-      <c r="M35" s="119" t="n"/>
-      <c r="N35" s="119" t="n"/>
-      <c r="O35" s="119" t="n"/>
-      <c r="P35" s="117" t="n"/>
-      <c r="Q35" s="117" t="n"/>
-      <c r="R35" s="117" t="n"/>
-      <c r="S35" s="119" t="n"/>
-      <c r="T35" s="117" t="n"/>
-      <c r="U35" s="117" t="n"/>
-      <c r="V35" s="117" t="n"/>
-      <c r="W35" s="117" t="n"/>
-      <c r="X35" s="117" t="n"/>
-      <c r="Y35" s="117" t="n"/>
-      <c r="Z35" s="117" t="n"/>
-      <c r="AA35" s="119" t="n"/>
-      <c r="AB35" s="119" t="n"/>
-      <c r="AC35" s="117" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="117" t="n"/>
-      <c r="B36" s="112" t="n"/>
-      <c r="C36" s="121" t="n"/>
-      <c r="D36" s="121" t="n"/>
-      <c r="E36" s="121" t="n"/>
-      <c r="F36" s="121" t="n"/>
-      <c r="G36" s="121" t="n"/>
-      <c r="H36" s="121" t="n"/>
-      <c r="I36" s="121" t="n"/>
-      <c r="J36" s="121" t="n"/>
-      <c r="K36" s="121" t="n"/>
-      <c r="L36" s="121" t="n"/>
-      <c r="M36" s="121" t="n"/>
-      <c r="N36" s="121" t="n"/>
-      <c r="O36" s="119" t="n"/>
-      <c r="P36" s="117" t="n"/>
-      <c r="Q36" s="117" t="n"/>
-      <c r="R36" s="117" t="n"/>
-      <c r="S36" s="119" t="n"/>
-      <c r="T36" s="117" t="n"/>
-      <c r="U36" s="117" t="n"/>
-      <c r="V36" s="117" t="n"/>
-      <c r="W36" s="117" t="n"/>
-      <c r="X36" s="117" t="n"/>
-      <c r="Y36" s="117" t="n"/>
-      <c r="Z36" s="117" t="n"/>
-      <c r="AA36" s="119" t="n"/>
-      <c r="AB36" s="119" t="n"/>
-      <c r="AC36" s="117" t="n"/>
+    <row r="28">
+      <c r="C28" s="110" t="n"/>
+      <c r="D28" s="110" t="n"/>
+      <c r="E28" s="110" t="n"/>
+      <c r="F28" s="110" t="n"/>
+      <c r="G28" s="110" t="n"/>
+      <c r="H28" s="110" t="n"/>
+      <c r="I28" s="111" t="n"/>
+      <c r="J28" s="110" t="n"/>
+      <c r="K28" s="111" t="n"/>
+      <c r="L28" s="17" t="n"/>
+      <c r="M28" s="111" t="n"/>
+      <c r="N28" s="17" t="n"/>
+      <c r="O28" s="17" t="n"/>
+      <c r="S28" s="17" t="n"/>
+      <c r="T28" s="8" t="n"/>
+      <c r="AA28" s="17" t="n"/>
+      <c r="AC28" s="8" t="n"/>
+    </row>
+    <row r="29" ht="16.5" customHeight="1">
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>4. SV MD　カウント方法</t>
+        </is>
+      </c>
+      <c r="L29" s="17" t="inlineStr">
+        <is>
+          <t>MAIN ITEM 原価計</t>
+        </is>
+      </c>
+      <c r="M29" s="112" t="inlineStr">
+        <is>
+          <t>Proportion</t>
+        </is>
+      </c>
+      <c r="N29" s="113" t="inlineStr">
+        <is>
+          <t>Submit</t>
+        </is>
+      </c>
+      <c r="O29" s="114" t="inlineStr">
+        <is>
+          <t>price/ea</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="14.25" customHeight="1">
+      <c r="B30" s="23" t="n"/>
+      <c r="C30" s="23" t="inlineStr">
+        <is>
+          <t>week</t>
+        </is>
+      </c>
+      <c r="D30" s="23" t="inlineStr">
+        <is>
+          <t>実働</t>
+        </is>
+      </c>
+      <c r="E30" s="23" t="inlineStr">
+        <is>
+          <t>休日</t>
+        </is>
+      </c>
+      <c r="F30" s="23" t="inlineStr">
+        <is>
+          <t>移動</t>
+        </is>
+      </c>
+      <c r="G30" s="115" t="inlineStr">
+        <is>
+          <t>計（C-MD）</t>
+        </is>
+      </c>
+      <c r="J30" s="116" t="n"/>
+      <c r="L30" s="17" t="n"/>
+      <c r="M30" s="117">
+        <f>IFERROR(L30/$L$33*$N$23,"")</f>
+        <v/>
+      </c>
+      <c r="N30" s="17" t="n"/>
+    </row>
+    <row r="31" ht="14.25" customHeight="1">
+      <c r="B31" s="56" t="inlineStr">
+        <is>
+          <t>SV A</t>
+        </is>
+      </c>
+      <c r="C31" s="56" t="n"/>
+      <c r="D31" s="56" t="n"/>
+      <c r="E31" s="56" t="n"/>
+      <c r="F31" s="56" t="n"/>
+      <c r="G31" s="118">
+        <f>SUM(D31:F31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="116" t="n"/>
+      <c r="L31" s="119" t="n"/>
+      <c r="M31" s="117">
+        <f>IFERROR(L31/$L$33*$N$23,"")</f>
+        <v/>
+      </c>
+      <c r="N31" s="17" t="n"/>
+    </row>
+    <row r="32" ht="14.25" customHeight="1">
+      <c r="B32" s="56" t="inlineStr">
+        <is>
+          <t>SV B</t>
+        </is>
+      </c>
+      <c r="C32" s="56" t="n"/>
+      <c r="D32" s="56" t="n"/>
+      <c r="E32" s="56" t="n"/>
+      <c r="F32" s="56" t="n"/>
+      <c r="G32" s="118">
+        <f>SUM(D32:F32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="116" t="n"/>
+      <c r="L32" s="119" t="n"/>
+      <c r="M32" s="117">
+        <f>IFERROR(L32/$L$33*$N$23,"")</f>
+        <v/>
+      </c>
+      <c r="N32" s="17" t="n"/>
+    </row>
+    <row r="33" ht="14.25" customHeight="1">
+      <c r="B33" s="56" t="inlineStr">
+        <is>
+          <t>SV C</t>
+        </is>
+      </c>
+      <c r="C33" s="56" t="n"/>
+      <c r="D33" s="56" t="n"/>
+      <c r="E33" s="56" t="n"/>
+      <c r="F33" s="56" t="n"/>
+      <c r="G33" s="118">
+        <f>SUM(D33:F33)</f>
+        <v/>
+      </c>
+      <c r="K33" s="111" t="n"/>
+      <c r="L33" s="17">
+        <f>SUM(L30:L32)</f>
+        <v/>
+      </c>
+      <c r="M33" s="17">
+        <f>SUM(M30:M32)</f>
+        <v/>
+      </c>
+      <c r="N33" s="17">
+        <f>SUM(N30:N32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34" ht="14.25" customHeight="1">
+      <c r="B34" s="56" t="inlineStr">
+        <is>
+          <t>SV D</t>
+        </is>
+      </c>
+      <c r="C34" s="56" t="n"/>
+      <c r="D34" s="56" t="n"/>
+      <c r="E34" s="56" t="n"/>
+      <c r="F34" s="56" t="n"/>
+      <c r="G34" s="118">
+        <f>SUM(D34:F34)</f>
+        <v/>
+      </c>
+      <c r="K34" s="8" t="n"/>
+      <c r="L34" s="17" t="n"/>
+      <c r="M34" s="17" t="n"/>
+      <c r="N34" s="17" t="n"/>
+    </row>
+    <row r="35" ht="14.25" customHeight="1">
+      <c r="B35" s="56" t="inlineStr">
+        <is>
+          <t>SV E</t>
+        </is>
+      </c>
+      <c r="C35" s="56" t="n"/>
+      <c r="D35" s="56" t="n"/>
+      <c r="E35" s="56" t="n"/>
+      <c r="F35" s="56" t="n"/>
+      <c r="G35" s="118">
+        <f>SUM(D35:F35)</f>
+        <v/>
+      </c>
+      <c r="K35" s="8" t="n"/>
+      <c r="L35" s="17" t="n"/>
+      <c r="M35" s="8" t="n"/>
+      <c r="N35" s="17" t="n"/>
+    </row>
+    <row r="36" ht="14.25" customHeight="1">
+      <c r="B36" s="56" t="inlineStr">
+        <is>
+          <t>SV F</t>
+        </is>
+      </c>
+      <c r="C36" s="56" t="n"/>
+      <c r="D36" s="56" t="n"/>
+      <c r="E36" s="56" t="n"/>
+      <c r="F36" s="56" t="n"/>
+      <c r="G36" s="118">
+        <f>SUM(D36:F36)</f>
+        <v/>
+      </c>
+      <c r="K36" s="8" t="n"/>
+      <c r="L36" s="17" t="n"/>
+      <c r="M36" s="17" t="n"/>
+      <c r="N36" s="17" t="n"/>
     </row>
     <row r="37">
-      <c r="C37" s="122" t="n"/>
-      <c r="D37" s="122" t="n"/>
-      <c r="E37" s="122" t="n"/>
-      <c r="F37" s="122" t="n"/>
-      <c r="G37" s="122" t="n"/>
-      <c r="H37" s="122" t="n"/>
-      <c r="I37" s="123" t="n"/>
-      <c r="J37" s="122" t="n"/>
-      <c r="K37" s="123" t="n"/>
-      <c r="L37" s="17" t="n"/>
-      <c r="M37" s="123" t="n"/>
-      <c r="N37" s="17" t="n"/>
-      <c r="O37" s="17" t="n"/>
-      <c r="S37" s="17" t="n"/>
-      <c r="T37" s="8" t="n"/>
-      <c r="AA37" s="17" t="n"/>
-      <c r="AC37" s="8" t="n"/>
-    </row>
-    <row r="38">
+      <c r="B37" s="56" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="G37" s="118">
+        <f>SUM(G31:G36)</f>
+        <v/>
+      </c>
+      <c r="M37" s="111" t="n"/>
+      <c r="N37" s="8" t="n"/>
+    </row>
+    <row r="38" ht="14.25" customHeight="1">
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t>4. SV MD　カウント方法</t>
-        </is>
-      </c>
-      <c r="L38" s="17" t="n"/>
-      <c r="N38" s="17" t="n"/>
-      <c r="O38" s="124" t="n"/>
+          <t>5. 残業</t>
+        </is>
+      </c>
+      <c r="C38" s="8" t="inlineStr">
+        <is>
+          <t>Offer</t>
+        </is>
+      </c>
+      <c r="D38" s="8" t="inlineStr">
+        <is>
+          <t>for calculation</t>
+        </is>
+      </c>
+      <c r="G38" s="120" t="n"/>
     </row>
     <row r="39">
-      <c r="B39" s="23" t="n"/>
-      <c r="C39" s="23" t="inlineStr">
-        <is>
-          <t>week</t>
-        </is>
-      </c>
-      <c r="D39" s="23" t="inlineStr">
-        <is>
-          <t>実働</t>
-        </is>
-      </c>
-      <c r="E39" s="23" t="inlineStr">
-        <is>
-          <t>休日</t>
-        </is>
-      </c>
-      <c r="F39" s="23" t="inlineStr">
-        <is>
-          <t>移動</t>
-        </is>
-      </c>
-      <c r="G39" s="125" t="inlineStr">
-        <is>
-          <t>計（C-MD）</t>
-        </is>
-      </c>
-      <c r="L39" s="17" t="n"/>
-      <c r="N39" s="17" t="n"/>
+      <c r="B39" s="121" t="inlineStr">
+        <is>
+          <t>月～金　C-md</t>
+        </is>
+      </c>
+      <c r="C39" s="122">
+        <f>D16*1000</f>
+        <v/>
+      </c>
+      <c r="D39" s="122">
+        <f>C39/8</f>
+        <v/>
+      </c>
+      <c r="E39" s="121" t="inlineStr">
+        <is>
+          <t>/hour</t>
+        </is>
+      </c>
+      <c r="G39" s="8" t="n"/>
+      <c r="R39" s="17" t="n"/>
+      <c r="T39" s="8" t="n"/>
+      <c r="Z39" s="17" t="n"/>
+      <c r="AA39" s="17" t="n"/>
+      <c r="AB39" s="8" t="n"/>
+      <c r="AC39" s="8" t="n"/>
     </row>
     <row r="40">
-      <c r="B40" s="56" t="n"/>
-      <c r="C40" s="56" t="n"/>
-      <c r="D40" s="56" t="n"/>
-      <c r="E40" s="56" t="n"/>
-      <c r="F40" s="56" t="n"/>
-      <c r="G40" s="126" t="n"/>
-      <c r="L40" s="17" t="n"/>
-      <c r="M40" s="17" t="n"/>
-      <c r="N40" s="17" t="n"/>
+      <c r="B40" s="56" t="inlineStr">
+        <is>
+          <t>月～金　17時～22時</t>
+        </is>
+      </c>
+      <c r="C40" s="46">
+        <f>ROUNDUP(D40,-3)</f>
+        <v/>
+      </c>
+      <c r="D40" s="46">
+        <f>$D$39*E40</f>
+        <v/>
+      </c>
+      <c r="E40" s="123" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="G40" s="8" t="n"/>
+      <c r="R40" s="17" t="n"/>
+      <c r="T40" s="8" t="n"/>
+      <c r="Z40" s="17" t="n"/>
+      <c r="AA40" s="17" t="n"/>
+      <c r="AB40" s="8" t="n"/>
+      <c r="AC40" s="8" t="n"/>
     </row>
     <row r="41">
-      <c r="B41" s="56" t="n"/>
-      <c r="C41" s="56" t="n"/>
-      <c r="D41" s="56" t="n"/>
-      <c r="E41" s="56" t="n"/>
-      <c r="F41" s="56" t="n"/>
-      <c r="G41" s="126" t="n"/>
-      <c r="M41" s="17" t="n"/>
-      <c r="N41" s="127" t="n"/>
+      <c r="B41" s="56" t="inlineStr">
+        <is>
+          <t>月～金　22時以降</t>
+        </is>
+      </c>
+      <c r="C41" s="46">
+        <f>ROUNDUP(D41,-3)</f>
+        <v/>
+      </c>
+      <c r="D41" s="46">
+        <f>$D$39*E41</f>
+        <v/>
+      </c>
+      <c r="E41" s="123" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G41" s="8" t="n"/>
+      <c r="R41" s="17" t="n"/>
+      <c r="T41" s="8" t="n"/>
+      <c r="Z41" s="17" t="n"/>
+      <c r="AA41" s="17" t="n"/>
+      <c r="AB41" s="8" t="n"/>
+      <c r="AC41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="B42" s="56" t="inlineStr">
         <is>
-          <t>SV A</t>
-        </is>
-      </c>
-      <c r="C42" s="56" t="n"/>
-      <c r="D42" s="56" t="n"/>
-      <c r="E42" s="56" t="n"/>
-      <c r="F42" s="56" t="n"/>
-      <c r="G42" s="126">
-        <f>SUM(D42:F42)</f>
-        <v/>
-      </c>
-      <c r="K42" s="123" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PTJ Proposal </t>
-        </is>
-      </c>
-      <c r="L42" s="8" t="n"/>
-      <c r="M42" s="123" t="n"/>
-      <c r="N42" s="17" t="n"/>
+          <t>土日、　8-17時</t>
+        </is>
+      </c>
+      <c r="C42" s="46">
+        <f>ROUNDUP(D42,-3)</f>
+        <v/>
+      </c>
+      <c r="D42" s="46">
+        <f>$D$39*E42</f>
+        <v/>
+      </c>
+      <c r="E42" s="123" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G42" s="8" t="n"/>
+      <c r="R42" s="17" t="n"/>
+      <c r="T42" s="8" t="n"/>
+      <c r="Z42" s="17" t="n"/>
+      <c r="AA42" s="17" t="n"/>
+      <c r="AB42" s="8" t="n"/>
+      <c r="AC42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="B43" s="56" t="inlineStr">
         <is>
-          <t>SV B</t>
-        </is>
-      </c>
-      <c r="C43" s="56" t="n"/>
-      <c r="D43" s="56" t="n"/>
-      <c r="E43" s="56" t="n"/>
-      <c r="F43" s="56" t="n"/>
-      <c r="G43" s="126">
-        <f>SUM(D43:F43)</f>
-        <v/>
-      </c>
-      <c r="K43" s="8" t="inlineStr">
-        <is>
-          <t>ME</t>
-        </is>
-      </c>
-      <c r="L43" s="17">
-        <f>N23</f>
-        <v/>
-      </c>
-      <c r="M43" s="17" t="n"/>
-      <c r="N43" s="17" t="n"/>
+          <t>土日、　17時～22時</t>
+        </is>
+      </c>
+      <c r="C43" s="46">
+        <f>ROUNDUP(D43,-3)</f>
+        <v/>
+      </c>
+      <c r="D43" s="46">
+        <f>$D$39*E43</f>
+        <v/>
+      </c>
+      <c r="E43" s="123" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="G43" s="8" t="n"/>
+      <c r="R43" s="17" t="n"/>
+      <c r="T43" s="8" t="n"/>
+      <c r="Z43" s="17" t="n"/>
+      <c r="AA43" s="17" t="n"/>
+      <c r="AB43" s="8" t="n"/>
+      <c r="AC43" s="8" t="n"/>
     </row>
     <row r="44">
-      <c r="B44" s="128" t="n"/>
-      <c r="C44" s="128" t="n"/>
-      <c r="D44" s="56" t="n"/>
-      <c r="E44" s="56" t="n"/>
-      <c r="F44" s="56" t="n"/>
-      <c r="G44" s="126" t="n"/>
-      <c r="K44" s="8" t="inlineStr">
-        <is>
-          <t>SV</t>
-        </is>
-      </c>
-      <c r="L44" s="17">
-        <f>N24</f>
-        <v/>
-      </c>
-      <c r="M44" s="8" t="n"/>
-      <c r="N44" s="17" t="n"/>
-    </row>
-    <row r="45">
-      <c r="B45" s="129" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="C45" s="129" t="n"/>
-      <c r="D45" s="129" t="n"/>
-      <c r="E45" s="129" t="n"/>
-      <c r="F45" s="129" t="n"/>
-      <c r="G45" s="130">
-        <f>SUM(G42:G44)</f>
-        <v/>
-      </c>
-      <c r="K45" s="8" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="L45" s="17">
-        <f>L43+L44</f>
-        <v/>
-      </c>
-      <c r="M45" s="17" t="n"/>
-      <c r="N45" s="17" t="n"/>
-    </row>
+      <c r="B44" s="85" t="inlineStr">
+        <is>
+          <t>土日、　22時以降</t>
+        </is>
+      </c>
+      <c r="C44" s="54">
+        <f>ROUNDUP(D44,-3)</f>
+        <v/>
+      </c>
+      <c r="D44" s="54">
+        <f>$D$39*E44</f>
+        <v/>
+      </c>
+      <c r="E44" s="124" t="n">
+        <v>2</v>
+      </c>
+      <c r="G44" s="8" t="n"/>
+      <c r="R44" s="17" t="n"/>
+      <c r="T44" s="8" t="n"/>
+      <c r="Z44" s="17" t="n"/>
+      <c r="AA44" s="17" t="n"/>
+      <c r="AB44" s="8" t="n"/>
+      <c r="AC44" s="8" t="n"/>
+    </row>
+    <row r="45"/>
     <row r="46">
-      <c r="M46" s="123" t="n"/>
-      <c r="N46" s="8" t="n"/>
-    </row>
-    <row r="47">
-      <c r="B47" s="8" t="inlineStr">
-        <is>
-          <t>5. 残業</t>
-        </is>
-      </c>
-      <c r="C47" s="8" t="inlineStr">
-        <is>
-          <t>Offer</t>
-        </is>
-      </c>
-      <c r="D47" s="8" t="inlineStr">
-        <is>
-          <t>for calculation</t>
-        </is>
-      </c>
-      <c r="G47" s="131" t="n"/>
-    </row>
-    <row r="48">
-      <c r="B48" s="132" t="inlineStr">
-        <is>
-          <t>月～金　C-md</t>
-        </is>
-      </c>
-      <c r="C48" s="133">
-        <f>D16*1000</f>
-        <v/>
-      </c>
-      <c r="D48" s="133">
-        <f>C48/8</f>
-        <v/>
-      </c>
-      <c r="E48" s="132" t="inlineStr">
-        <is>
-          <t>/hour</t>
-        </is>
-      </c>
-      <c r="G48" s="8" t="n"/>
-      <c r="R48" s="17" t="n"/>
-      <c r="T48" s="8" t="n"/>
-      <c r="Z48" s="17" t="n"/>
-      <c r="AA48" s="17" t="n"/>
-      <c r="AB48" s="8" t="n"/>
-      <c r="AC48" s="8" t="n"/>
-    </row>
-    <row r="49">
-      <c r="B49" s="56" t="inlineStr">
-        <is>
-          <t>月～金　17時～22時</t>
-        </is>
-      </c>
-      <c r="C49" s="46">
-        <f>ROUNDUP(D49,-3)</f>
-        <v/>
-      </c>
-      <c r="D49" s="46">
-        <f>$D$48*E49</f>
-        <v/>
-      </c>
-      <c r="E49" s="134" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="G49" s="8" t="n"/>
-      <c r="R49" s="17" t="n"/>
-      <c r="T49" s="8" t="n"/>
-      <c r="Z49" s="17" t="n"/>
-      <c r="AA49" s="17" t="n"/>
-      <c r="AB49" s="8" t="n"/>
-      <c r="AC49" s="8" t="n"/>
-    </row>
-    <row r="50">
-      <c r="B50" s="56" t="inlineStr">
-        <is>
-          <t>月～金　22時以降</t>
-        </is>
-      </c>
-      <c r="C50" s="46">
-        <f>ROUNDUP(D50,-3)</f>
-        <v/>
-      </c>
-      <c r="D50" s="46">
-        <f>$D$48*E50</f>
-        <v/>
-      </c>
-      <c r="E50" s="134" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G50" s="8" t="n"/>
-      <c r="R50" s="17" t="n"/>
-      <c r="T50" s="8" t="n"/>
-      <c r="Z50" s="17" t="n"/>
-      <c r="AA50" s="17" t="n"/>
-      <c r="AB50" s="8" t="n"/>
-      <c r="AC50" s="8" t="n"/>
-    </row>
-    <row r="51">
-      <c r="B51" s="56" t="inlineStr">
-        <is>
-          <t>土日、　8-17時</t>
-        </is>
-      </c>
-      <c r="C51" s="46">
-        <f>ROUNDUP(D51,-3)</f>
-        <v/>
-      </c>
-      <c r="D51" s="46">
-        <f>$D$48*E51</f>
-        <v/>
-      </c>
-      <c r="E51" s="134" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G51" s="8" t="n"/>
-      <c r="R51" s="17" t="n"/>
-      <c r="T51" s="8" t="n"/>
-      <c r="Z51" s="17" t="n"/>
-      <c r="AA51" s="17" t="n"/>
-      <c r="AB51" s="8" t="n"/>
-      <c r="AC51" s="8" t="n"/>
-    </row>
-    <row r="52">
-      <c r="B52" s="56" t="inlineStr">
-        <is>
-          <t>土日、　17時～22時</t>
-        </is>
-      </c>
-      <c r="C52" s="46">
-        <f>ROUNDUP(D52,-3)</f>
-        <v/>
-      </c>
-      <c r="D52" s="46">
-        <f>$D$48*E52</f>
-        <v/>
-      </c>
-      <c r="E52" s="134" t="n">
-        <v>1.75</v>
-      </c>
-      <c r="G52" s="8" t="n"/>
-      <c r="R52" s="17" t="n"/>
-      <c r="T52" s="8" t="n"/>
-      <c r="Z52" s="17" t="n"/>
-      <c r="AA52" s="17" t="n"/>
-      <c r="AB52" s="8" t="n"/>
-      <c r="AC52" s="8" t="n"/>
-    </row>
-    <row r="53">
-      <c r="B53" s="85" t="inlineStr">
-        <is>
-          <t>土日、　22時以降</t>
-        </is>
-      </c>
-      <c r="C53" s="54">
-        <f>ROUNDUP(D53,-3)</f>
-        <v/>
-      </c>
-      <c r="D53" s="54">
-        <f>$D$48*E53</f>
-        <v/>
-      </c>
-      <c r="E53" s="135" t="n">
-        <v>2</v>
-      </c>
-      <c r="G53" s="8" t="n"/>
-      <c r="R53" s="17" t="n"/>
-      <c r="T53" s="8" t="n"/>
-      <c r="Z53" s="17" t="n"/>
-      <c r="AA53" s="17" t="n"/>
-      <c r="AB53" s="8" t="n"/>
-      <c r="AC53" s="8" t="n"/>
-    </row>
-    <row r="55">
-      <c r="O55" s="136" t="n"/>
+      <c r="O46" s="125" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="4">
+    <mergeCell ref="J30:K30"/>
     <mergeCell ref="D4:E4"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="J31:K31"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ptj-internal-estimate: K15 RC remark가 엑셀 수식으로 오인되던 문제 수정
- build_template_v2.py: K15 라벨에서 선행 '=' 제거 ('= まとめ CONTI' → 'まとめ CONTI ... 합')
- nemae.py: K15 RC remark는 자동입력하지 않음을 주석으로 명시
- nemae_template.xlsx: 수정된 스크립트로 재빌드
</commit_message>
<xml_diff>
--- a/ptj-internal-estimate/assets/nemae_template.xlsx
+++ b/ptj-internal-estimate/assets/nemae_template.xlsx
@@ -809,9 +809,10 @@
       <c r="J15" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="8">
-        <f> まとめ CONTI(WA/EX/PS)</f>
-        <v/>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>まとめ CONTI(WA/EX/PS) 합</t>
+        </is>
       </c>
     </row>
     <row r="16">

</xml_diff>